<commit_message>
Sperre und Quellenluecke im Regelkern, damit Summenfehler und unbekannte Taetigkeiten nicht still entschieden werden.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
+++ b/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regeln" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelregister" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schwellen nach Jahr" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offene Punkte" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tätigkeitskatalog" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abgabesätze" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pauschalen nach Jahr" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textbausteine" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tätigkeitsabgrenzung" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Regeln" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Regelregister" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Schwellen nach Jahr" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Offene Punkte" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tätigkeitskatalog" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Abgabesätze" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Pauschalen nach Jahr" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Textbausteine" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Tätigkeitsabgrenzung" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Regelregister'!$A$1:$J$23</definedName>
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -16280,6 +16280,1196 @@
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>rechtsform.kein_entgelt</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ggmbh</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rechtsform</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>R-138</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Ableitung: gGmbH ist eine GmbH</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>rechtsform.kein_entgelt</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>oeffentlich</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Rechtsform</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>F-006</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Oeffentliche Stelle ist kein selbststaendiger Kuenstler</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>sperre.summenabweichung</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: gedruckte Summe weicht von der Positionssumme ab</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>sperre.ust_inkonsistent</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Umsatzsteuer ist nicht konsistent</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>sperre.positionsnummer</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Positionsnummer doppelt</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>sperre.rechnungsbetrag</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Rechnungsbetrag ist nicht Netto plus Umsatzsteuer</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>sperre.negative_summe</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: negative Gesamtsumme</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sperre.ust_satz</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Umsatzsteuersatz ohne Hinweis</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>sperre.netto_fehlt</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Nettosumme fehlt</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>sperre.doppelzahlung</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Zahlung doppelt erfasst</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>auslage.nachgewiesen</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>auslage</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Paragraf 18 Abs. 1 Nr. 2 SGB IV: nachgewiesene Auslage</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>gesang</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>tanz</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>choreografie</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>regie</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>komposition</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>fotografie</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>schauspiel</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>dirigent</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>bühnenbild</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>straßenkünstler</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>dj</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>moderation</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>redaktion</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>textbeitrag</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>illustration</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>podcast</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>videojournalismus</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>grafikdesign</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>kameramann</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>werbeflyer</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>texterstellung</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>eigenwerbung</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
@@ -24282,60 +25472,60 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>T-76</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Fotomodell, Model, Mannequin (Modellhonorar)</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Grenzfall</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D47" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>fotomodell; modellhonorar; mannequin; dressman; laufstegmodel</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>Fotomodelle nennt KSK-Info 06 nicht; das Modell ordnete sie live als darstellende Kunst ein.</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>R-137</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Abschn. 1</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Entwurf – vom Steuerberater zu prüfen</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>Neu 15.10.2026 (Alltagstest AT-2026-024, live f6a5d1a: Modellhonorar 800 € still mitgezählt, 382,20 € statt 343,00 €). Frage an den Steuerberater (Q-36).</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="4" t="inlineStr">
         <is>
           <t>prüfen</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M47" s="4" t="inlineStr">
         <is>
           <t>Abgrenzung offen.</t>
         </is>

</xml_diff>

<commit_message>
Erfahrungs-Suite misst Sperre, Quellenluecke und Belege, damit die gefundenen Loecher nicht zurueckkommen.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
+++ b/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -16286,1190 +16286,1400 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>rechtsform.kein_entgelt</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>ggmbh</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Rechtsform</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>R-138</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Ableitung: gGmbH ist eine GmbH</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>rechtsform.kein_entgelt</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>oeffentlich</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Rechtsform</t>
         </is>
       </c>
-      <c r="E28" t="n">
+      <c r="E28" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>F-006</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>Oeffentliche Stelle ist kein selbststaendiger Kuenstler</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>sperre.summenabweichung</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: gedruckte Summe weicht von der Positionssumme ab</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>sperre.ust_inkonsistent</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E30" t="n">
+      <c r="E30" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Umsatzsteuer ist nicht konsistent</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>sperre.positionsnummer</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Positionsnummer doppelt</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>sperre.rechnungsbetrag</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Rechnungsbetrag ist nicht Netto plus Umsatzsteuer</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>sperre.negative_summe</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: negative Gesamtsumme</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>sperre.ust_satz</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Umsatzsteuersatz ohne Hinweis</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>sperre.netto_fehlt</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Nettosumme fehlt</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>sperre.doppelzahlung</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Zahlung doppelt erfasst</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>auslage.nachgewiesen</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>auslage</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="E37" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I37" s="4" t="inlineStr">
         <is>
           <t>Paragraf 18 Abs. 1 Nr. 2 SGB IV: nachgewiesene Auslage</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J37" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>gesang</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E38" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J38" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>tanz</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J39" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>choreografie</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E40" t="n">
+      <c r="E40" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I40" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>regie</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>komposition</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E42" t="n">
+      <c r="E42" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>fotografie</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>schauspiel</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J44" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>dirigent</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J45" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>bühnenbild</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E46" t="n">
+      <c r="E46" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J46" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>straßenkünstler</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>dj</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E48" t="n">
+      <c r="E48" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>moderation</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H49" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I49" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J49" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>feature</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I50" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J50" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>redaktion</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I51" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="J51" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>textbeitrag</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E52" t="n">
+      <c r="E52" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J52" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>illustration</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I53" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J53" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>podcast</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I54" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="J54" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>videojournalismus</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="I55" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>grafikdesign</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H56" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I56" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="J56" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>kameramann</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>werbeflyer</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E58" t="n">
+      <c r="E58" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I58" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="J58" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>texterstellung</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E59" t="n">
+      <c r="E59" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="H59" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="I59" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="J59" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>eigenwerbung</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E60" t="n">
+      <c r="E60" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I60" s="4" t="inlineStr">
         <is>
           <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>sperre.manipulation</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: nachtraeglich geaenderte Zeile</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>sperre.paragraph19</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>sperre</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Kleinunternehmer und Umsatzsteuer widersprechen sich</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>sperre.toleranz</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Euro</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Rundungsdifferenz ueber 1 Cent</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>rechtsform.kein_entgelt</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>se</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Rechtsform</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>R-138</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Ableitung: die SE ist einer AG gleichgestellt</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>taetigkeit.ausgeschlossen</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>beratung</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>F-006</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Beratung ist keine kuenstlerische oder publizistische Leistung</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>taetigkeit.ausgeschlossen</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>buchhaltung</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>F-006</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Buchhaltung ist keine kuenstlerische oder publizistische Leistung</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>

</xml_diff>

<commit_message>
Dokumentpruefungen und Cent-Toleranz aus dem Register, Konzert nur als Leistung.
Widersprueche in der Rechnung sperren ohne Abgabe, ein Cent bleibt ein Hinweis, und eine blosse Erwaehnung eines Konzerts zaehlt nicht als Musikleistung.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
+++ b/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -16433,7 +16433,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>sperre</t>
+          <t>doppelte Positionsnummer — Zeilensplitting oder Duplikat prüfen</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -16468,7 +16468,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>sperre</t>
+          <t>Rechenprobe brutto</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -16503,7 +16503,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>sperre</t>
+          <t>Negative Gesamtsumme ohne Stornorechnung</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -17476,210 +17476,350 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>sperre.manipulation</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>sperre</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="H61" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="I61" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: nachtraeglich geaenderte Zeile</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="J61" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>sperre.paragraph19</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>sperre</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Widerspruch §19 UStG — Rechnung prüfen</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E62" t="n">
+      <c r="E62" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H62" s="4" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="I62" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Kleinunternehmer und Umsatzsteuer widersprechen sich</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="J62" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>sperre.toleranz</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>Euro</t>
         </is>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="H63" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="I63" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Rundungsdifferenz ueber 1 Cent</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="J63" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>rechtsform.kein_entgelt</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>se</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Rechtsform</t>
         </is>
       </c>
-      <c r="E64" t="n">
+      <c r="E64" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>R-138</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="I64" s="4" t="inlineStr">
         <is>
           <t>Ableitung: die SE ist einer AG gleichgestellt</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="J64" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.ausgeschlossen</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>beratung</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" s="4" t="inlineStr">
         <is>
           <t>F-006</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I65" s="4" t="inlineStr">
         <is>
           <t>Beratung ist keine kuenstlerische oder publizistische Leistung</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="J65" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.ausgeschlossen</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>buchhaltung</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E66" t="n">
+      <c r="E66" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H66" s="4" t="inlineStr">
         <is>
           <t>F-006</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="I66" s="4" t="inlineStr">
         <is>
           <t>Buchhaltung ist keine kuenstlerische oder publizistische Leistung</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>sperre.toleranz_ab</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Euro</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Rundungsdifferenz ab 2 Cent ist eine Sperre</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>sperre.toleranz_hinweis</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Rundungsdifferenz 1 ct, rechnerisch unbedeutend</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: bis 1 Cent kein Sperrgrund</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>offen.skonto</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Ist der Skonto in der Summe enthalten?</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: Skonto-Abzug unklar, keine Sperre</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>offen.storno</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Storno im selben Jahr: Saldierung ist zu prüfen</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: negative Summe mit Storno bleibt offen</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
@@ -23471,10 +23611,14 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>kompon; jingle; arrangeur; arrangement; musiker; sänger; audio-design; sounddesign; sound-design; discjockey; dj; liedermacher; songwriter; musik; konzert</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr"/>
+          <t>kompon; jingle; arrangeur; arrangement; musiker; sänger; audio-design; sounddesign; sound-design; discjockey; dj; liedermacher; songwriter; musik; konzert; konzertauftritt; konzerthonorar; konzertgage; konzertmitwirkung; live-konzert; musikdarbietung; musikauffuehrung</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>konzert und musik zaehlen nur, wenn sie die Leistung benennen. Blosse Erwaehnung (des Konzerts) ist kein Treffer.</t>
+        </is>
+      </c>
       <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Register aus den KSK-Infos fuellen, ohne stille Grenzfälle.
Webdesign und Maskenbild am Theater sind belegt und entschieden. Übersetzung, Unterricht und Ausland bleiben Rückfrage, weil die Quellen den Einzelfall offen lassen.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
+++ b/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -17686,140 +17686,3785 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>sperre.toleranz_ab</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>0.02</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>Euro</t>
         </is>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H67" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I67" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Rundungsdifferenz ab 2 Cent ist eine Sperre</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="J67" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>sperre.toleranz_hinweis</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>Rundungsdifferenz 1 ct, rechnerisch unbedeutend</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E68" t="n">
+      <c r="E68" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
+      <c r="I68" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: bis 1 Cent kein Sperrgrund</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="J68" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>offen.skonto</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>Ist der Skonto in der Summe enthalten?</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I69" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: Skonto-Abzug unklar, keine Sperre</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="J69" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>offen.storno</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>Storno im selben Jahr: Saldierung ist zu prüfen</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E70" t="n">
+      <c r="E70" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="H70" s="4" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
+      <c r="I70" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: negative Summe mit Storno bleibt offen</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>clown</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: clown</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>comedian</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: comedian</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>kabarettist</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: kabarettist</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>komiker</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: komiker</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>illustrator</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: illustrator</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>journalist</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: journalist</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>kostümbildner</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: kostümbildner</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>grafiker</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: grafiker</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>bildhauer</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: bildhauer</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>choreograph</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: choreograph</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>fotograf</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: fotograf</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>maler</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: maler</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>maskenbilder</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: maskenbilder</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>redakteur</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: redakteur</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>musiker</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: musiker</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>sänger</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: sänger</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>schriftsteller</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: schriftsteller</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>sprecher</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: sprecher</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>synchronsprecher</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: synchronsprecher</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>puppenspieler</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: puppenspieler</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>marionettenspieler</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: marionettenspieler</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>pantomime</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: pantomime</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>zauberer</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: zauberer</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>visagist</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: visagist</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>instrumentalsolist</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: instrumentalsolist</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>webdesigner</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: webdesigner</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>web-designer</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: web-designer</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>webdesign</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: webdesign</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>maskenbildner</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: maskenbildner</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>publizist</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: publizist</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>reporter</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: reporter</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>kritiker</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: kritiker</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>herausgeber</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: herausgeber</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>liedermacher</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: liedermacher</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>songwriter</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: songwriter</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>texter</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: texter</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>layouter</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: layouter</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>comiczeichner</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: comiczeichner</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>karikaturist</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: karikaturist</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>rezitator</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: rezitator</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>drehbuchautor</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: drehbuchautor</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>filmemacher</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: filmemacher</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>regisseur</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: regisseur</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>komponist</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: komponist</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>autor</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: autor</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>pressefotograf</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: pressefotograf</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>werbefotograf</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: werbefotograf</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>game-designer</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Info-06</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: game-designer</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>taetigkeit.synonym</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>corporate-design</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Info-02</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>KSK-Info 02, S. 1, Abschnitt 4: Corporate-Design ist eine Design-Leistung, die vom KSVG erfasst ist.</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>übersetzung</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote * (Besonderheiten, schriftlich bei der KSK anfragen). Literarisch oder Fachübersetzung entscheidet der Einzelfall.</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>übersetzer</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>übersetzerin</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>uebersetzung</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>uebersetzer</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>kunstunterricht</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 1: Künstler ist auch, wer Kunst lehrt; S. 2 nennt Lehrer für künstlerische Tätigkeiten. Ob die konkrete Stunde nur Unterricht ist, sagt der Katalog nicht.</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>gesangsunterricht</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 3 nennt Musiklehrer, nicht die einzelne Gesangsstunde. Darbietung oder pädagogische Vermittlung bleibt Einzelfall.</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>stimmcoaching</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>KSK-Info 06 nennt Sprecherzieher und Musiklehrer, nicht Stimmcoaching. Pädagogische Vermittlung oder Darbietung ist nicht entschieden.</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>lektor</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 2 führt Lektor auf. Info 09, S. 4, Abschnitt 3.2: bei mehreren Leistungsanteilen entscheidet der überwiegende Teil. Kein Automatismus.</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>taetigkeit.offen</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>lektorat</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Info-06-Offen</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>KSK-Info 06, S. 2 führt Lektor auf. Info 09, S. 4, Abschnitt 3.2: bei mehreren Leistungsanteilen entscheidet der überwiegende Teil. Kein Automatismus.</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ausland.kuenstler</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>ausländisch</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Info-22</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>KSK-Info 22, Stand 10.2025, S. 1-2, Abschn. 2 und 6: Abgabe auf selbständige ausländische Künstler ja, abhängige Beschäftigung und A1-Bescheinigung nein. Status nach deutschem Recht ist zu klären.</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ausland.kuenstler</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>auslaendisch</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Info-22</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>KSK-Info 22, Stand 10.2025, S. 1-2, Abschn. 6: Die KSK prüft selbständige oder abhängige Tätigkeit nach deutschem Recht. Bescheinigungen des Auslands sind kein Nachweis.</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>ausland.kuenstler</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>auslandssachverhalt</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Info-22</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>KSK-Info 22, Stand 10.2025, S. 1 Abschn. 2: Auslandsbezug hebt die Abgabe nicht auf. Ob ein abhängiges Beschäftigungsverhältnis vorliegt, ist zu klären.</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>gemeinnuetzig</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>gemeinnützig</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Info-23</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>KSK-Info 23, Stand 01.2026, S. 1 Abschn. 2: Gemeinnützigkeit befreit nicht und begründet die Abgabe nicht allein. Befreiungstatbestände sind nicht vorgesehen.</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>gemeinnuetzig</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>gemeinnuetzig</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Info-23</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>KSK-Info 23, Stand 01.2026, S. 1 Abschn. 2: Gemeinnützigkeit befreit nicht und begründet die Abgabe nicht allein.</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>auftraggeber.kommune</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>stadt</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Info-11</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>KSK-Info 11, Stand der Datei, S. 1 Abschn. 1-2: Städte, Landkreise und Gemeinden können abgabepflichtig sein. Das ist kein Ausschluss wie eine Zahlung an eine öffentliche Körperschaft als Empfänger.</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>auftraggeber.kommune</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>landkreis</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Info-11</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>KSK-Info 11, Stand der Datei, S. 1 Abschn. 1-2: Städte, Landkreise und Gemeinden können abgabepflichtig sein. Das ist kein Ausschluss wie eine Zahlung an eine öffentliche Körperschaft als Empfänger.</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>auftraggeber.kommune</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>gemeinde</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Info-11</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>KSK-Info 11, Stand der Datei, S. 1 Abschn. 1-2: Städte, Landkreise und Gemeinden können abgabepflichtig sein. Das ist kein Ausschluss wie eine Zahlung an eine öffentliche Körperschaft als Empfänger.</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>gesellschafter.gmbh</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>gesellschafter</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Gesellschafter</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>KSK-Merkblatt Gesellschafter einer GmbH, S. 1-2: Mitarbeitender Gesellschafter ist nur bei maßgeblichem Einfluss selbständig. Künstlerischer Anteil und Oberleitung prüft die KSK. BSG 16.04.1998, B 3 KR 7/97 R, im Merkblatt zitiert.</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>musikverein.schueler_unter</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Schüler</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Info-12-P1</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>KSK-Info 12, Stand 01.2026, S. 2 Punkt 1: nicht mehr als 20 Schüler, dem Grunde nach keine Abgabepflicht nach § 24 Abs. 1 Nr. 9 KSVG.</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>musikverein.schueler_mitte</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>vermutung</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Info-12-P2</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>KSK-Info 12, Stand 01.2026, S. 2 Punkt 2: mehr als 20 und weniger als 61 Schüler, Vermutung keine Abgabepflicht nach § 24 Abs. 1 Nr. 9, wenn kein Ausbilder über der Übungsleiterpauschale liegt.</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>entgelt.ausgenommen</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>gema</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>KSVG-25</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>KSVG § 25 Abs. 2: Entgelte für Nutzungsrechte an Verwertungsgesellschaften sind ausgenommen (Gesetzestext im Repo, Seite 9).</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>entgelt.ausgenommen</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>verwertungsgesellschaft</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>KSVG-25</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>KSVG § 25 Abs. 2 Nr. 1: Entgelte an Verwertungsgesellschaften für urheberrechtliche Nutzungsrechte gehören nicht zum Entgelt.</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>entgelt.ausgenommen</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>verwertung</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>KSVG-25</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>KSVG § 25 Abs. 2 Nr. 1: Zahlung wegen Verwertung an eine Verwertungsgesellschaft, nicht schon jede Verlagsleistung.</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>entgelt.ausgenommen</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>musikverlag</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>KSVG-25</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>KSK-Checkliste Verlage und KSVG § 25 Abs. 2 Nr. 1: Lizenzzahlung, die als Verwertung ausgewiesen ist. Ein Verlag ist nicht schon deshalb eine Verwertungsgesellschaft.</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>reise</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>fahrt</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>übernachtung</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>uebernachtung</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>verpflegung</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>bewirtung</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>auslage</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>materialkosten</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>notenmappe</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>notenkauf</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>kostenübernahme</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>auslage.auch_ohne_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>notenkauf</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Weiterberechnete Auslage Noten oder Kostenübernahme, wie bisher im Register auslage.nachgewiesen geführt.</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>auslage.auch_ohne_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>kostenübernahme</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Weiterberechnete Auslage Noten oder Kostenübernahme, wie bisher im Register auslage.nachgewiesen geführt.</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>auslage.auch_ohne_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>notenmappe</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Weiterberechnete Auslage Noten oder Kostenübernahme, wie bisher im Register auslage.nachgewiesen geführt.</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>auslage</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>materialkosten</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>reise</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>fahrt</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>übernachtung</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>uebernachtung</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>auslage.ohne_beleg_offen</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>verpflegung</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>porto</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>versand</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>kopierkosten</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>rahmen</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>plakat</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>scanner-miete</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>notenmaterial</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>

</xml_diff>

<commit_message>
Zahlenquellen an das Regelregister angleichen.
Historische Abgabesaetze und die geteilte 450-Euro-Grenze stehen jetzt mit derselben Fundstelle wie im Register. Eigenwerbung ist kein Taetigkeitssynonym mehr.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
+++ b/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J174"/>
+  <dimension ref="A1:J177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -17443,7 +17443,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>taetigkeit.synonym</t>
+          <t>szenarien.eigenwerbung</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -17461,12 +17461,12 @@
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>KSVG-24-2</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>Quellenluecke: ohne Katalogtreffer keine automatische Entscheidung</t>
+          <t>KSVG § 24 Abs. 2 Satz 1 Nummer 1. Eigenwerbung ist ein Verwerter-Szenario, keine Tätigkeit.</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr">
@@ -17826,3645 +17826,3750 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>clown</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H71" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
+      <c r="I71" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: clown</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="J71" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>comedian</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E72" t="n">
+      <c r="E72" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="H72" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="I72" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: comedian</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="J72" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>kabarettist</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E73" t="n">
+      <c r="E73" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H73" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I73" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: kabarettist</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="J73" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>komiker</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H74" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="I74" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: komiker</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="J74" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>illustrator</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="H75" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I75" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: illustrator</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="J75" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>journalist</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="H76" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="I76" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: journalist</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="J76" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>kostümbildner</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H77" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
+      <c r="I77" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: kostümbildner</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="J77" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>grafiker</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E78" t="n">
+      <c r="E78" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H78" t="inlineStr">
+      <c r="H78" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr">
+      <c r="I78" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: grafiker</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="J78" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>bildhauer</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E79" t="n">
+      <c r="E79" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H79" t="inlineStr">
+      <c r="H79" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
+      <c r="I79" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: bildhauer</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="J79" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>choreograph</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E80" t="n">
+      <c r="E80" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="H80" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
+      <c r="I80" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: choreograph</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="J80" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>fotograf</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E81" t="n">
+      <c r="E81" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="H81" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
+      <c r="I81" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: fotograf</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="J81" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>maler</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E82" t="n">
+      <c r="E82" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="H82" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
+      <c r="I82" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: maler</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr">
+      <c r="J82" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>maskenbilder</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E83" t="n">
+      <c r="E83" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H83" t="inlineStr">
+      <c r="H83" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr">
+      <c r="I83" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: maskenbilder</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="J83" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>redakteur</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E84" t="n">
+      <c r="E84" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H84" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr">
+      <c r="I84" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 2, Katalog künstlerische/publizistische Tätigkeiten: redakteur</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="J84" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>musiker</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E85" t="n">
+      <c r="E85" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H85" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
+      <c r="I85" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: musiker</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="J85" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>sänger</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E86" t="n">
+      <c r="E86" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H86" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
+      <c r="I86" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: sänger</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="J86" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>schriftsteller</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E87" t="n">
+      <c r="E87" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="H87" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
+      <c r="I87" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: schriftsteller</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr">
+      <c r="J87" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>sprecher</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E88" t="n">
+      <c r="E88" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="H88" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr">
+      <c r="I88" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: sprecher</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr">
+      <c r="J88" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>synchronsprecher</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E89" t="n">
+      <c r="E89" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="H89" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr">
+      <c r="I89" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: synchronsprecher</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="J89" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>puppenspieler</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E90" t="n">
+      <c r="E90" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="H90" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
+      <c r="I90" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: puppenspieler</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="J90" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="4" t="inlineStr">
         <is>
           <t>marionettenspieler</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E91" t="n">
+      <c r="E91" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="H91" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
+      <c r="I91" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: marionettenspieler</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr">
+      <c r="J91" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="4" t="inlineStr">
         <is>
           <t>pantomime</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E92" t="n">
+      <c r="E92" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H92" t="inlineStr">
+      <c r="H92" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr">
+      <c r="I92" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: pantomime</t>
         </is>
       </c>
-      <c r="J92" t="inlineStr">
+      <c r="J92" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>zauberer</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E93" t="n">
+      <c r="E93" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="H93" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr">
+      <c r="I93" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: zauberer</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr">
+      <c r="J93" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>visagist</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E94" t="n">
+      <c r="E94" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H94" t="inlineStr">
+      <c r="H94" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr">
+      <c r="I94" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: visagist</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr">
+      <c r="J94" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>instrumentalsolist</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C95" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E95" t="n">
+      <c r="E95" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H95" t="inlineStr">
+      <c r="H95" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
+      <c r="I95" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: instrumentalsolist</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr">
+      <c r="J95" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>webdesigner</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E96" t="n">
+      <c r="E96" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H96" t="inlineStr">
+      <c r="H96" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr">
+      <c r="I96" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: webdesigner</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr">
+      <c r="J96" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>web-designer</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E97" t="n">
+      <c r="E97" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H97" t="inlineStr">
+      <c r="H97" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr">
+      <c r="I97" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: web-designer</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr">
+      <c r="J97" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>webdesign</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E98" t="n">
+      <c r="E98" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H98" t="inlineStr">
+      <c r="H98" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr">
+      <c r="I98" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: webdesign</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr">
+      <c r="J98" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="4" t="inlineStr">
         <is>
           <t>maskenbildner</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E99" t="n">
+      <c r="E99" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H99" t="inlineStr">
+      <c r="H99" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr">
+      <c r="I99" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: maskenbildner</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr">
+      <c r="J99" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>publizist</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C100" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E100" t="n">
+      <c r="E100" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H100" t="inlineStr">
+      <c r="H100" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr">
+      <c r="I100" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: publizist</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr">
+      <c r="J100" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>reporter</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E101" t="n">
+      <c r="E101" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H101" t="inlineStr">
+      <c r="H101" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr">
+      <c r="I101" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: reporter</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr">
+      <c r="J101" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>kritiker</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E102" t="n">
+      <c r="E102" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H102" t="inlineStr">
+      <c r="H102" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr">
+      <c r="I102" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: kritiker</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr">
+      <c r="J102" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B103" s="4" t="inlineStr">
         <is>
           <t>herausgeber</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C103" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E103" t="n">
+      <c r="E103" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H103" t="inlineStr">
+      <c r="H103" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr">
+      <c r="I103" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: herausgeber</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr">
+      <c r="J103" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
+      <c r="A104" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>liedermacher</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C104" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E104" t="n">
+      <c r="E104" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H104" t="inlineStr">
+      <c r="H104" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr">
+      <c r="I104" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: liedermacher</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr">
+      <c r="J104" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B105" s="4" t="inlineStr">
         <is>
           <t>songwriter</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C105" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E105" t="n">
+      <c r="E105" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H105" t="inlineStr">
+      <c r="H105" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr">
+      <c r="I105" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: songwriter</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr">
+      <c r="J105" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
+      <c r="A106" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B106" s="4" t="inlineStr">
         <is>
           <t>texter</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C106" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E106" t="n">
+      <c r="E106" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H106" t="inlineStr">
+      <c r="H106" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr">
+      <c r="I106" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: texter</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr">
+      <c r="J106" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
+      <c r="A107" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B107" s="4" t="inlineStr">
         <is>
           <t>layouter</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C107" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E107" t="n">
+      <c r="E107" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H107" t="inlineStr">
+      <c r="H107" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr">
+      <c r="I107" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: layouter</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr">
+      <c r="J107" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
+      <c r="A108" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B108" s="4" t="inlineStr">
         <is>
           <t>comiczeichner</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C108" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E108" t="n">
+      <c r="E108" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H108" t="inlineStr">
+      <c r="H108" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr">
+      <c r="I108" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: comiczeichner</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr">
+      <c r="J108" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
+      <c r="A109" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B109" s="4" t="inlineStr">
         <is>
           <t>karikaturist</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C109" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E109" t="n">
+      <c r="E109" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H109" t="inlineStr">
+      <c r="H109" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr">
+      <c r="I109" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: karikaturist</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr">
+      <c r="J109" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
+      <c r="A110" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B110" s="4" t="inlineStr">
         <is>
           <t>rezitator</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C110" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E110" t="n">
+      <c r="E110" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H110" t="inlineStr">
+      <c r="H110" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr">
+      <c r="I110" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: rezitator</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr">
+      <c r="J110" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
+      <c r="A111" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>drehbuchautor</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C111" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E111" t="n">
+      <c r="E111" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H111" t="inlineStr">
+      <c r="H111" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr">
+      <c r="I111" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: drehbuchautor</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr">
+      <c r="J111" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
+      <c r="A112" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B112" s="4" t="inlineStr">
         <is>
           <t>filmemacher</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C112" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E112" t="n">
+      <c r="E112" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H112" t="inlineStr">
+      <c r="H112" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
+      <c r="I112" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: filmemacher</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr">
+      <c r="J112" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
+      <c r="A113" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>regisseur</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C113" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E113" t="n">
+      <c r="E113" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H113" t="inlineStr">
+      <c r="H113" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr">
+      <c r="I113" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: regisseur</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr">
+      <c r="J113" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
+      <c r="A114" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>komponist</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C114" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E114" t="n">
+      <c r="E114" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H114" t="inlineStr">
+      <c r="H114" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
+      <c r="I114" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: komponist</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="J114" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
+      <c r="A115" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>autor</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E115" t="n">
+      <c r="E115" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H115" t="inlineStr">
+      <c r="H115" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr">
+      <c r="I115" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: autor</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr">
+      <c r="J115" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>pressefotograf</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C116" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E116" t="n">
+      <c r="E116" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H116" t="inlineStr">
+      <c r="H116" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr">
+      <c r="I116" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: pressefotograf</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr">
+      <c r="J116" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
+      <c r="A117" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B117" s="4" t="inlineStr">
         <is>
           <t>werbefotograf</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C117" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E117" t="n">
+      <c r="E117" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H117" t="inlineStr">
+      <c r="H117" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr">
+      <c r="I117" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: werbefotograf</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr">
+      <c r="J117" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
+      <c r="A118" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>game-designer</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C118" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E118" t="n">
+      <c r="E118" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H118" t="inlineStr">
+      <c r="H118" s="4" t="inlineStr">
         <is>
           <t>Info-06</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr">
+      <c r="I118" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, Stand 09.2025, S. 3, Katalog künstlerische/publizistische Tätigkeiten: game-designer</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr">
+      <c r="J118" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
+      <c r="A119" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.synonym</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B119" s="4" t="inlineStr">
         <is>
           <t>corporate-design</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
+      <c r="C119" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E119" t="n">
+      <c r="E119" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H119" t="inlineStr">
+      <c r="H119" s="4" t="inlineStr">
         <is>
           <t>Info-02</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr">
+      <c r="I119" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 02, S. 1, Abschnitt 4: Corporate-Design ist eine Design-Leistung, die vom KSVG erfasst ist.</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr">
+      <c r="J119" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
+      <c r="A120" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>übersetzung</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C120" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E120" t="n">
+      <c r="E120" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H120" t="inlineStr">
+      <c r="H120" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr">
+      <c r="I120" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote * (Besonderheiten, schriftlich bei der KSK anfragen). Literarisch oder Fachübersetzung entscheidet der Einzelfall.</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr">
+      <c r="J120" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr">
+      <c r="A121" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>übersetzer</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E121" t="n">
+      <c r="E121" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H121" t="inlineStr">
+      <c r="H121" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr">
+      <c r="I121" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr">
+      <c r="J121" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr">
+      <c r="A122" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B122" s="4" t="inlineStr">
         <is>
           <t>übersetzerin</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C122" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E122" t="n">
+      <c r="E122" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H122" t="inlineStr">
+      <c r="H122" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr">
+      <c r="I122" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr">
+      <c r="J122" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr">
+      <c r="A123" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B123" s="4" t="inlineStr">
         <is>
           <t>uebersetzung</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C123" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E123" t="n">
+      <c r="E123" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H123" t="inlineStr">
+      <c r="H123" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr">
+      <c r="I123" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr">
+      <c r="J123" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr">
+      <c r="A124" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
+      <c r="B124" s="4" t="inlineStr">
         <is>
           <t>uebersetzer</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
+      <c r="C124" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E124" t="n">
+      <c r="E124" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H124" t="inlineStr">
+      <c r="H124" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr">
+      <c r="I124" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 3: Übersetzer/Bearbeiter mit Fussnote *. Keine stille Wahl zwischen literarisch und Fachübersetzung.</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr">
+      <c r="J124" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr">
+      <c r="A125" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
+      <c r="B125" s="4" t="inlineStr">
         <is>
           <t>kunstunterricht</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
+      <c r="C125" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E125" t="n">
+      <c r="E125" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H125" t="inlineStr">
+      <c r="H125" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr">
+      <c r="I125" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 1: Künstler ist auch, wer Kunst lehrt; S. 2 nennt Lehrer für künstlerische Tätigkeiten. Ob die konkrete Stunde nur Unterricht ist, sagt der Katalog nicht.</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr">
+      <c r="J125" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr">
+      <c r="A126" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B126" s="4" t="inlineStr">
         <is>
           <t>gesangsunterricht</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C126" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E126" t="n">
+      <c r="E126" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H126" t="inlineStr">
+      <c r="H126" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr">
+      <c r="I126" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 3 nennt Musiklehrer, nicht die einzelne Gesangsstunde. Darbietung oder pädagogische Vermittlung bleibt Einzelfall.</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr">
+      <c r="J126" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
+      <c r="A127" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B127" s="4" t="inlineStr">
         <is>
           <t>stimmcoaching</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C127" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E127" t="n">
+      <c r="E127" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H127" t="inlineStr">
+      <c r="H127" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr">
+      <c r="I127" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06 nennt Sprecherzieher und Musiklehrer, nicht Stimmcoaching. Pädagogische Vermittlung oder Darbietung ist nicht entschieden.</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr">
+      <c r="J127" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr">
+      <c r="A128" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B128" s="4" t="inlineStr">
         <is>
           <t>lektor</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
+      <c r="C128" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E128" t="n">
+      <c r="E128" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H128" t="inlineStr">
+      <c r="H128" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr">
+      <c r="I128" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 2 führt Lektor auf. Info 09, S. 4, Abschnitt 3.2: bei mehreren Leistungsanteilen entscheidet der überwiegende Teil. Kein Automatismus.</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr">
+      <c r="J128" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr">
+      <c r="A129" s="4" t="inlineStr">
         <is>
           <t>taetigkeit.offen</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
+      <c r="B129" s="4" t="inlineStr">
         <is>
           <t>lektorat</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C129" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E129" t="n">
+      <c r="E129" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H129" t="inlineStr">
+      <c r="H129" s="4" t="inlineStr">
         <is>
           <t>Info-06-Offen</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr">
+      <c r="I129" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 06, S. 2 führt Lektor auf. Info 09, S. 4, Abschnitt 3.2: bei mehreren Leistungsanteilen entscheidet der überwiegende Teil. Kein Automatismus.</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr">
+      <c r="J129" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr">
+      <c r="A130" s="4" t="inlineStr">
         <is>
           <t>ausland.kuenstler</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
+      <c r="B130" s="4" t="inlineStr">
         <is>
           <t>ausländisch</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C130" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E130" t="n">
+      <c r="E130" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H130" t="inlineStr">
+      <c r="H130" s="4" t="inlineStr">
         <is>
           <t>Info-22</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr">
+      <c r="I130" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 22, Stand 10.2025, S. 1-2, Abschn. 2 und 6: Abgabe auf selbständige ausländische Künstler ja, abhängige Beschäftigung und A1-Bescheinigung nein. Status nach deutschem Recht ist zu klären.</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr">
+      <c r="J130" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr">
+      <c r="A131" s="4" t="inlineStr">
         <is>
           <t>ausland.kuenstler</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
+      <c r="B131" s="4" t="inlineStr">
         <is>
           <t>auslaendisch</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C131" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E131" t="n">
+      <c r="E131" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H131" t="inlineStr">
+      <c r="H131" s="4" t="inlineStr">
         <is>
           <t>Info-22</t>
         </is>
       </c>
-      <c r="I131" t="inlineStr">
+      <c r="I131" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 22, Stand 10.2025, S. 1-2, Abschn. 6: Die KSK prüft selbständige oder abhängige Tätigkeit nach deutschem Recht. Bescheinigungen des Auslands sind kein Nachweis.</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr">
+      <c r="J131" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr">
+      <c r="A132" s="4" t="inlineStr">
         <is>
           <t>ausland.kuenstler</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
+      <c r="B132" s="4" t="inlineStr">
         <is>
           <t>auslandssachverhalt</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
+      <c r="C132" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E132" t="n">
+      <c r="E132" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H132" t="inlineStr">
+      <c r="H132" s="4" t="inlineStr">
         <is>
           <t>Info-22</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr">
+      <c r="I132" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 22, Stand 10.2025, S. 1 Abschn. 2: Auslandsbezug hebt die Abgabe nicht auf. Ob ein abhängiges Beschäftigungsverhältnis vorliegt, ist zu klären.</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr">
+      <c r="J132" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr">
+      <c r="A133" s="4" t="inlineStr">
         <is>
           <t>gemeinnuetzig</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B133" s="4" t="inlineStr">
         <is>
           <t>gemeinnützig</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
+      <c r="C133" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E133" t="n">
+      <c r="E133" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H133" t="inlineStr">
+      <c r="H133" s="4" t="inlineStr">
         <is>
           <t>Info-23</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr">
+      <c r="I133" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 23, Stand 01.2026, S. 1 Abschn. 2: Gemeinnützigkeit befreit nicht und begründet die Abgabe nicht allein. Befreiungstatbestände sind nicht vorgesehen.</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr">
+      <c r="J133" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr">
+      <c r="A134" s="4" t="inlineStr">
         <is>
           <t>gemeinnuetzig</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
+      <c r="B134" s="4" t="inlineStr">
         <is>
           <t>gemeinnuetzig</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
+      <c r="C134" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E134" t="n">
+      <c r="E134" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H134" t="inlineStr">
+      <c r="H134" s="4" t="inlineStr">
         <is>
           <t>Info-23</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr">
+      <c r="I134" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 23, Stand 01.2026, S. 1 Abschn. 2: Gemeinnützigkeit befreit nicht und begründet die Abgabe nicht allein.</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr">
+      <c r="J134" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr">
+      <c r="A135" s="4" t="inlineStr">
         <is>
           <t>auftraggeber.kommune</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
+      <c r="B135" s="4" t="inlineStr">
         <is>
           <t>stadt</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C135" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E135" t="n">
+      <c r="E135" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H135" t="inlineStr">
+      <c r="H135" s="4" t="inlineStr">
         <is>
           <t>Info-11</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr">
+      <c r="I135" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 11, Stand der Datei, S. 1 Abschn. 1-2: Städte, Landkreise und Gemeinden können abgabepflichtig sein. Das ist kein Ausschluss wie eine Zahlung an eine öffentliche Körperschaft als Empfänger.</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr">
+      <c r="J135" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr">
+      <c r="A136" s="4" t="inlineStr">
         <is>
           <t>auftraggeber.kommune</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
+      <c r="B136" s="4" t="inlineStr">
         <is>
           <t>landkreis</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
+      <c r="C136" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E136" t="n">
+      <c r="E136" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H136" t="inlineStr">
+      <c r="H136" s="4" t="inlineStr">
         <is>
           <t>Info-11</t>
         </is>
       </c>
-      <c r="I136" t="inlineStr">
+      <c r="I136" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 11, Stand der Datei, S. 1 Abschn. 1-2: Städte, Landkreise und Gemeinden können abgabepflichtig sein. Das ist kein Ausschluss wie eine Zahlung an eine öffentliche Körperschaft als Empfänger.</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr">
+      <c r="J136" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr">
+      <c r="A137" s="4" t="inlineStr">
         <is>
           <t>auftraggeber.kommune</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B137" s="4" t="inlineStr">
         <is>
           <t>gemeinde</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
+      <c r="C137" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E137" t="n">
+      <c r="E137" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H137" t="inlineStr">
+      <c r="H137" s="4" t="inlineStr">
         <is>
           <t>Info-11</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr">
+      <c r="I137" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 11, Stand der Datei, S. 1 Abschn. 1-2: Städte, Landkreise und Gemeinden können abgabepflichtig sein. Das ist kein Ausschluss wie eine Zahlung an eine öffentliche Körperschaft als Empfänger.</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr">
+      <c r="J137" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr">
+      <c r="A138" s="4" t="inlineStr">
         <is>
           <t>gesellschafter.gmbh</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
+      <c r="B138" s="4" t="inlineStr">
         <is>
           <t>gesellschafter</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C138" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E138" t="n">
+      <c r="E138" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H138" t="inlineStr">
+      <c r="H138" s="4" t="inlineStr">
         <is>
           <t>Gesellschafter</t>
         </is>
       </c>
-      <c r="I138" t="inlineStr">
+      <c r="I138" s="4" t="inlineStr">
         <is>
           <t>KSK-Merkblatt Gesellschafter einer GmbH, S. 1-2: Mitarbeitender Gesellschafter ist nur bei maßgeblichem Einfluss selbständig. Künstlerischer Anteil und Oberleitung prüft die KSK. BSG 16.04.1998, B 3 KR 7/97 R, im Merkblatt zitiert.</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr">
+      <c r="J138" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr">
+      <c r="A139" s="4" t="inlineStr">
         <is>
           <t>musikverein.schueler_unter</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
+      <c r="B139" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
+      <c r="C139" s="4" t="inlineStr">
         <is>
           <t>Schüler</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr">
+      <c r="D139" s="4" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="E139" t="n">
+      <c r="E139" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H139" t="inlineStr">
+      <c r="H139" s="4" t="inlineStr">
         <is>
           <t>Info-12-P1</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr">
+      <c r="I139" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 12, Stand 01.2026, S. 2 Punkt 1: nicht mehr als 20 Schüler, dem Grunde nach keine Abgabepflicht nach § 24 Abs. 1 Nr. 9 KSVG.</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr">
+      <c r="J139" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr">
+      <c r="A140" s="4" t="inlineStr">
         <is>
           <t>musikverein.schueler_mitte</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
+      <c r="B140" s="4" t="inlineStr">
         <is>
           <t>vermutung</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C140" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E140" t="n">
+      <c r="E140" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H140" t="inlineStr">
+      <c r="H140" s="4" t="inlineStr">
         <is>
           <t>Info-12-P2</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr">
+      <c r="I140" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 12, Stand 01.2026, S. 2 Punkt 2: mehr als 20 und weniger als 61 Schüler, Vermutung keine Abgabepflicht nach § 24 Abs. 1 Nr. 9, wenn kein Ausbilder über der Übungsleiterpauschale liegt.</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr">
+      <c r="J140" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr">
+      <c r="A141" s="4" t="inlineStr">
         <is>
           <t>entgelt.ausgenommen</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
+      <c r="B141" s="4" t="inlineStr">
         <is>
           <t>gema</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
+      <c r="C141" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E141" t="n">
+      <c r="E141" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H141" t="inlineStr">
+      <c r="H141" s="4" t="inlineStr">
         <is>
           <t>KSVG-25</t>
         </is>
       </c>
-      <c r="I141" t="inlineStr">
+      <c r="I141" s="4" t="inlineStr">
         <is>
           <t>KSVG § 25 Abs. 2: Entgelte für Nutzungsrechte an Verwertungsgesellschaften sind ausgenommen (Gesetzestext im Repo, Seite 9).</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr">
+      <c r="J141" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr">
+      <c r="A142" s="4" t="inlineStr">
         <is>
           <t>entgelt.ausgenommen</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
+      <c r="B142" s="4" t="inlineStr">
         <is>
           <t>verwertungsgesellschaft</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
+      <c r="C142" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E142" t="n">
+      <c r="E142" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H142" t="inlineStr">
+      <c r="H142" s="4" t="inlineStr">
         <is>
           <t>KSVG-25</t>
         </is>
       </c>
-      <c r="I142" t="inlineStr">
+      <c r="I142" s="4" t="inlineStr">
         <is>
           <t>KSVG § 25 Abs. 2 Nr. 1: Entgelte an Verwertungsgesellschaften für urheberrechtliche Nutzungsrechte gehören nicht zum Entgelt.</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr">
+      <c r="J142" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr">
+      <c r="A143" s="4" t="inlineStr">
         <is>
           <t>entgelt.ausgenommen</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
+      <c r="B143" s="4" t="inlineStr">
         <is>
           <t>verwertung</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
+      <c r="C143" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E143" t="n">
+      <c r="E143" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H143" t="inlineStr">
+      <c r="H143" s="4" t="inlineStr">
         <is>
           <t>KSVG-25</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr">
+      <c r="I143" s="4" t="inlineStr">
         <is>
           <t>KSVG § 25 Abs. 2 Nr. 1: Zahlung wegen Verwertung an eine Verwertungsgesellschaft, nicht schon jede Verlagsleistung.</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr">
+      <c r="J143" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr">
+      <c r="A144" s="4" t="inlineStr">
         <is>
           <t>entgelt.ausgenommen</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
+      <c r="B144" s="4" t="inlineStr">
         <is>
           <t>musikverlag</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
+      <c r="C144" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E144" t="n">
+      <c r="E144" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H144" t="inlineStr">
+      <c r="H144" s="4" t="inlineStr">
         <is>
           <t>KSVG-25</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr">
+      <c r="I144" s="4" t="inlineStr">
         <is>
           <t>KSK-Checkliste Verlage und KSVG § 25 Abs. 2 Nr. 1: Lizenzzahlung, die als Verwertung ausgewiesen ist. Ein Verlag ist nicht schon deshalb eine Verwertungsgesellschaft.</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr">
+      <c r="J144" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr">
+      <c r="A145" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
+      <c r="B145" s="4" t="inlineStr">
         <is>
           <t>reise</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
+      <c r="C145" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E145" t="n">
+      <c r="E145" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H145" t="inlineStr">
+      <c r="H145" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr">
+      <c r="I145" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr">
+      <c r="J145" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr">
+      <c r="A146" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
+      <c r="B146" s="4" t="inlineStr">
         <is>
           <t>fahrt</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C146" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E146" t="n">
+      <c r="E146" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H146" t="inlineStr">
+      <c r="H146" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr">
+      <c r="I146" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr">
+      <c r="J146" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr">
+      <c r="A147" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
+      <c r="B147" s="4" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
+      <c r="C147" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E147" t="n">
+      <c r="E147" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H147" t="inlineStr">
+      <c r="H147" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr">
+      <c r="I147" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr">
+      <c r="J147" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr">
+      <c r="A148" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+      <c r="B148" s="4" t="inlineStr">
         <is>
           <t>übernachtung</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
+      <c r="C148" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E148" t="n">
+      <c r="E148" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H148" t="inlineStr">
+      <c r="H148" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr">
+      <c r="I148" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr">
+      <c r="J148" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
+      <c r="A149" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B149" s="4" t="inlineStr">
         <is>
           <t>uebernachtung</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C149" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E149" t="n">
+      <c r="E149" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H149" t="inlineStr">
+      <c r="H149" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr">
+      <c r="I149" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr">
+      <c r="J149" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr">
+      <c r="A150" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B150" s="4" t="inlineStr">
         <is>
           <t>verpflegung</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
+      <c r="C150" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E150" t="n">
+      <c r="E150" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H150" t="inlineStr">
+      <c r="H150" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr">
+      <c r="I150" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr">
+      <c r="J150" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
+      <c r="A151" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B151" s="4" t="inlineStr">
         <is>
           <t>bewirtung</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C151" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E151" t="n">
+      <c r="E151" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H151" t="inlineStr">
+      <c r="H151" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr">
+      <c r="I151" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr">
+      <c r="J151" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr">
+      <c r="A152" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B152" s="4" t="inlineStr">
         <is>
           <t>auslage</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
+      <c r="C152" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E152" t="n">
+      <c r="E152" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H152" t="inlineStr">
+      <c r="H152" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I152" t="inlineStr">
+      <c r="I152" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr">
+      <c r="J152" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr">
+      <c r="A153" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
+      <c r="B153" s="4" t="inlineStr">
         <is>
           <t>materialkosten</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
+      <c r="C153" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E153" t="n">
+      <c r="E153" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H153" t="inlineStr">
+      <c r="H153" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I153" t="inlineStr">
+      <c r="I153" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr">
+      <c r="J153" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
+      <c r="A154" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="4" t="inlineStr">
         <is>
           <t>notenmappe</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C154" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E154" t="n">
+      <c r="E154" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H154" t="inlineStr">
+      <c r="H154" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I154" t="inlineStr">
+      <c r="I154" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr">
+      <c r="J154" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
+      <c r="A155" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B155" s="4" t="inlineStr">
         <is>
           <t>notenkauf</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C155" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E155" t="n">
+      <c r="E155" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H155" t="inlineStr">
+      <c r="H155" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr">
+      <c r="I155" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr">
+      <c r="J155" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr">
+      <c r="A156" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B156" s="4" t="inlineStr">
         <is>
           <t>kostenübernahme</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
+      <c r="C156" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E156" t="n">
+      <c r="E156" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H156" t="inlineStr">
+      <c r="H156" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I156" t="inlineStr">
+      <c r="I156" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 und KSK-Info 10: nur die dort genannten nachgewiesenen Nebenleistungen fallen aus der Bemessung. Beleg erforderlich.</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr">
+      <c r="J156" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr">
+      <c r="A157" s="4" t="inlineStr">
         <is>
           <t>auslage.auch_ohne_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B157" s="4" t="inlineStr">
         <is>
           <t>notenkauf</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C157" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E157" t="n">
+      <c r="E157" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H157" t="inlineStr">
+      <c r="H157" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr">
+      <c r="I157" s="4" t="inlineStr">
         <is>
           <t>Weiterberechnete Auslage Noten oder Kostenübernahme, wie bisher im Register auslage.nachgewiesen geführt.</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr">
+      <c r="J157" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr">
+      <c r="A158" s="4" t="inlineStr">
         <is>
           <t>auslage.auch_ohne_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr">
+      <c r="B158" s="4" t="inlineStr">
         <is>
           <t>kostenübernahme</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
+      <c r="C158" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E158" t="n">
+      <c r="E158" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H158" t="inlineStr">
+      <c r="H158" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I158" t="inlineStr">
+      <c r="I158" s="4" t="inlineStr">
         <is>
           <t>Weiterberechnete Auslage Noten oder Kostenübernahme, wie bisher im Register auslage.nachgewiesen geführt.</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr">
+      <c r="J158" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
+      <c r="A159" s="4" t="inlineStr">
         <is>
           <t>auslage.auch_ohne_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B159" s="4" t="inlineStr">
         <is>
           <t>notenmappe</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C159" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E159" t="n">
+      <c r="E159" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H159" t="inlineStr">
+      <c r="H159" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I159" t="inlineStr">
+      <c r="I159" s="4" t="inlineStr">
         <is>
           <t>Weiterberechnete Auslage Noten oder Kostenübernahme, wie bisher im Register auslage.nachgewiesen geführt.</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr">
+      <c r="J159" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr">
+      <c r="A160" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr">
+      <c r="B160" s="4" t="inlineStr">
         <is>
           <t>auslage</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
+      <c r="C160" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E160" t="n">
+      <c r="E160" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H160" t="inlineStr">
+      <c r="H160" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr">
+      <c r="I160" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J160" t="inlineStr">
+      <c r="J160" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr">
+      <c r="A161" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr">
+      <c r="B161" s="4" t="inlineStr">
         <is>
           <t>materialkosten</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
+      <c r="C161" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E161" t="n">
+      <c r="E161" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H161" t="inlineStr">
+      <c r="H161" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I161" t="inlineStr">
+      <c r="I161" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr">
+      <c r="J161" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr">
+      <c r="A162" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
+      <c r="B162" s="4" t="inlineStr">
         <is>
           <t>reise</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C162" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E162" t="n">
+      <c r="E162" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H162" t="inlineStr">
+      <c r="H162" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I162" t="inlineStr">
+      <c r="I162" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J162" t="inlineStr">
+      <c r="J162" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr">
+      <c r="A163" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B163" s="4" t="inlineStr">
         <is>
           <t>fahrt</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C163" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E163" t="n">
+      <c r="E163" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H163" t="inlineStr">
+      <c r="H163" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr">
+      <c r="I163" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr">
+      <c r="J163" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr">
+      <c r="A164" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B164" s="4" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C164" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E164" t="n">
+      <c r="E164" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H164" t="inlineStr">
+      <c r="H164" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr">
+      <c r="I164" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr">
+      <c r="J164" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr">
+      <c r="A165" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
+      <c r="B165" s="4" t="inlineStr">
         <is>
           <t>übernachtung</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C165" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E165" t="n">
+      <c r="E165" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H165" t="inlineStr">
+      <c r="H165" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I165" t="inlineStr">
+      <c r="I165" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr">
+      <c r="J165" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr">
+      <c r="A166" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr">
+      <c r="B166" s="4" t="inlineStr">
         <is>
           <t>uebernachtung</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C166" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E166" t="n">
+      <c r="E166" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H166" t="inlineStr">
+      <c r="H166" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I166" t="inlineStr">
+      <c r="I166" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J166" t="inlineStr">
+      <c r="J166" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr">
+      <c r="A167" s="4" t="inlineStr">
         <is>
           <t>auslage.ohne_beleg_offen</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
+      <c r="B167" s="4" t="inlineStr">
         <is>
           <t>verpflegung</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
+      <c r="C167" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E167" t="n">
+      <c r="E167" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H167" t="inlineStr">
+      <c r="H167" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I167" t="inlineStr">
+      <c r="I167" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1 und Info 10: ohne Nachweis keine Ausnahme. Verpflegung zusätzlich an verpflegung.stunden_grenze und verpflegung.stunden_ganztag im Register gebunden.</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr">
+      <c r="J167" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr">
+      <c r="A168" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr">
+      <c r="B168" s="4" t="inlineStr">
         <is>
           <t>porto</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr">
+      <c r="C168" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E168" t="n">
+      <c r="E168" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H168" t="inlineStr">
+      <c r="H168" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr">
+      <c r="I168" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J168" t="inlineStr">
+      <c r="J168" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr">
+      <c r="A169" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr">
+      <c r="B169" s="4" t="inlineStr">
         <is>
           <t>versand</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
+      <c r="C169" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E169" t="n">
+      <c r="E169" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H169" t="inlineStr">
+      <c r="H169" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I169" t="inlineStr">
+      <c r="I169" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J169" t="inlineStr">
+      <c r="J169" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr">
+      <c r="A170" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B170" s="4" t="inlineStr">
         <is>
           <t>kopierkosten</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C170" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E170" t="n">
+      <c r="E170" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H170" t="inlineStr">
+      <c r="H170" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I170" t="inlineStr">
+      <c r="I170" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr">
+      <c r="J170" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr">
+      <c r="A171" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr">
+      <c r="B171" s="4" t="inlineStr">
         <is>
           <t>rahmen</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
+      <c r="C171" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E171" t="n">
+      <c r="E171" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H171" t="inlineStr">
+      <c r="H171" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I171" t="inlineStr">
+      <c r="I171" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr">
+      <c r="J171" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr">
+      <c r="A172" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B172" t="inlineStr">
+      <c r="B172" s="4" t="inlineStr">
         <is>
           <t>plakat</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr">
+      <c r="C172" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E172" t="n">
+      <c r="E172" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H172" t="inlineStr">
+      <c r="H172" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr">
+      <c r="I172" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J172" t="inlineStr">
+      <c r="J172" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr">
+      <c r="A173" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B173" s="4" t="inlineStr">
         <is>
           <t>scanner-miete</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
+      <c r="C173" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E173" t="n">
+      <c r="E173" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H173" t="inlineStr">
+      <c r="H173" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I173" t="inlineStr">
+      <c r="I173" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J173" t="inlineStr">
+      <c r="J173" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr">
+      <c r="A174" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B174" s="4" t="inlineStr">
         <is>
           <t>notenmaterial</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C174" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E174" t="n">
+      <c r="E174" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H174" t="inlineStr">
+      <c r="H174" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr">
+      <c r="I174" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr">
+      <c r="J174" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>offen.waehrung</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Fremdwährung ohne Umrechnungsnachweis — Kurs und Nachweis vorlegen</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Testfall L-23: Euro-Betrag und Umrechnungsgrundlage klären; keine erfundene Euro-Summe. Eine Umrechnungsregel ist in der Quellenbasis nicht belegt.</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>auslage.mit_beleg_ausgenommen</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>verpflegungsmehraufwand</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>KSVEntgV-1</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>auslage.gehoert_zum_entgelt</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>plakatrahmen</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Info-10</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>

</xml_diff>

<commit_message>
Dokumentpruefung vor der Entscheidung.
Strukturierte Suite-Felder speisen Summenprobe, Positionsnummer, Paragraf 19, negative Summe und Cent-Toleranz. Zwei Rechtsformen sperren, statt still eine zu waehlen.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
+++ b/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J177"/>
+  <dimension ref="A1:J178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -21471,105 +21471,140 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr">
+      <c r="A175" s="4" t="inlineStr">
         <is>
           <t>offen.waehrung</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr">
+      <c r="B175" s="4" t="inlineStr">
         <is>
           <t>Fremdwährung ohne Umrechnungsnachweis — Kurs und Nachweis vorlegen</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C175" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E175" t="n">
+      <c r="E175" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H175" t="inlineStr">
+      <c r="H175" s="4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="I175" t="inlineStr">
+      <c r="I175" s="4" t="inlineStr">
         <is>
           <t>Testfall L-23: Euro-Betrag und Umrechnungsgrundlage klären; keine erfundene Euro-Summe. Eine Umrechnungsregel ist in der Quellenbasis nicht belegt.</t>
         </is>
       </c>
-      <c r="J175" t="inlineStr">
+      <c r="J175" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr">
+      <c r="A176" s="4" t="inlineStr">
         <is>
           <t>auslage.mit_beleg_ausgenommen</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr">
+      <c r="B176" s="4" t="inlineStr">
         <is>
           <t>verpflegungsmehraufwand</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr">
+      <c r="C176" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E176" t="n">
+      <c r="E176" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H176" t="inlineStr">
+      <c r="H176" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV-1</t>
         </is>
       </c>
-      <c r="I176" t="inlineStr">
+      <c r="I176" s="4" t="inlineStr">
         <is>
           <t>KSVEntgV § 1 Nr. 1: nachgewiesene Reisekosten innerhalb der Grenzen des § 3 Nr. 16 EStG zählen nicht. KSK-Info 10, S. 2.</t>
         </is>
       </c>
-      <c r="J176" t="inlineStr">
+      <c r="J176" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr">
+      <c r="A177" s="4" t="inlineStr">
         <is>
           <t>auslage.gehoert_zum_entgelt</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B177" s="4" t="inlineStr">
         <is>
           <t>plakatrahmen</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C177" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E177" t="n">
+      <c r="E177" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H177" t="inlineStr">
+      <c r="H177" s="4" t="inlineStr">
         <is>
           <t>Info-10</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr">
+      <c r="I177" s="4" t="inlineStr">
         <is>
           <t>KSK-Info 10, S. 1: Auslagen und Nebenkosten, die dem Künstler vergütet werden, gehören zum Entgelt. Ausnahme nur Umsatzsteuer, Verwertungsgesellschaft, Reise und übliche Bewirtung.</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr">
+      <c r="J177" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>sperre.rechtsform</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Widerspruch der Rechtsform: mehrere Gesellschaftsformen im selben Dokument</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Rechenprobe A2/A3: widerspruechliche Angaben zur Rechtsform, keine stille Wahl</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>

</xml_diff>

<commit_message>
USt-Mischsatz und oeffentliche Stelle im Kern pruefen.
Der Schluessel kommt zuerst aus der Umgebung, sonst aus der Datei, und wird nicht mitgeschrieben.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
+++ b/regelwerk/Regelkatalog_24_KSVG_Entwurf.xlsx
@@ -15138,7 +15138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J178"/>
+  <dimension ref="A1:J182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -21576,35 +21576,175 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr">
+      <c r="A178" s="4" t="inlineStr">
         <is>
           <t>sperre.rechtsform</t>
         </is>
       </c>
-      <c r="B178" t="inlineStr">
+      <c r="B178" s="4" t="inlineStr">
         <is>
           <t>Widerspruch der Rechtsform: mehrere Gesellschaftsformen im selben Dokument</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr">
+      <c r="C178" s="4" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E178" t="n">
+      <c r="E178" s="4" t="n">
         <v>2015</v>
       </c>
-      <c r="H178" t="inlineStr">
+      <c r="H178" s="4" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr">
+      <c r="I178" s="4" t="inlineStr">
         <is>
           <t>Rechenprobe A2/A3: widerspruechliche Angaben zur Rechtsform, keine stille Wahl</t>
         </is>
       </c>
-      <c r="J178" t="inlineStr">
+      <c r="J178" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="4" t="inlineStr">
+        <is>
+          <t>ust.satz</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>Prozent</t>
+        </is>
+      </c>
+      <c r="E179" s="4" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H179" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t>UStG § 12 Abs. 2: ermäßigter Steuersatz 7 Prozent. Der Satz steht im Register, nicht im Code.</t>
+        </is>
+      </c>
+      <c r="J179" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>ust.satz</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>Prozent</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H180" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I180" s="4" t="inlineStr">
+        <is>
+          <t>UStG § 12 Abs. 1: Regelsteuersatz 19 Prozent. Der Satz steht im Register, nicht im Code.</t>
+        </is>
+      </c>
+      <c r="J180" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t>sperre.ust_mischsatz</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>USt-Rechenprobe, Mischsaetze</t>
+        </is>
+      </c>
+      <c r="C181" s="4" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E181" s="4" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H181" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="I181" s="4" t="inlineStr">
+        <is>
+          <t>§ 25 Abs. 1 KSVG: die Abgabe bemisst sich nach dem Entgelt. Rechenprobe: ausgewiesene Umsatzsteuer passt zu keinem Satz und die Summe zu keinem einheitlichen Satz.</t>
+        </is>
+      </c>
+      <c r="J181" s="4" t="inlineStr">
+        <is>
+          <t>Entwurf – vom Steuerberater zu prüfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>offen.oeffentliche_stelle</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>Öffentliche Stelle als Verwerter: Info 11/16, Rückfrage ob die Verwertereigenschaft in Betracht kommt.</t>
+        </is>
+      </c>
+      <c r="C182" s="4" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E182" s="4" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H182" s="4" t="inlineStr">
+        <is>
+          <t>Info-11</t>
+        </is>
+      </c>
+      <c r="I182" s="4" t="inlineStr">
+        <is>
+          <t>KSK-Info 11, S. 1 Abschn. 1-2: Städte, Landkreise und Gemeinden können abgabepflichtig sein. KSK-Info 16, Stand 09.2025: Abgabepflicht öffentlich-rechtlicher Institutionen. Keine stille Ausnahme wie eine Zahlung an eine Kapitalgesellschaft.</t>
+        </is>
+      </c>
+      <c r="J182" s="4" t="inlineStr">
         <is>
           <t>Entwurf – vom Steuerberater zu prüfen</t>
         </is>

</xml_diff>